<commit_message>
feat: Implement data parsing, generate pillar progress charts, and display thematic summaries with maturity levels.
</commit_message>
<xml_diff>
--- a/data/DRM Rapid Screening Tool - Cameroon (false).xlsx
+++ b/data/DRM Rapid Screening Tool - Cameroon (false).xlsx
@@ -913,9 +913,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="31.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="40.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="23.67"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="4" width="9.49"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="10" min="9" style="3" width="6.71"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="11" min="11" style="4" width="17.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="4" width="9.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="3" width="6.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="4" width="17.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="28.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="20.57"/>
@@ -1074,7 +1074,7 @@
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="18" t="str">
         <f aca="false">IF(COUNTBLANK(E15:E60)&gt;0,_xlfn.CONCAT("Please complete the assessment to proceed. Remaining questions: ",COUNTBLANK(E15:E60)), _xlfn.TEXTJOIN("&amp;",FALSE(),K15:K60))</f>
-        <v>Q1;Yes;1&amp;Q2;Yes;1&amp;Q3;Yes;1&amp;Q4;Partially;1&amp;Q5;Yes;1&amp;Q6;No;1&amp;Q7;Yes;1&amp;Q8;Yes;1&amp;Q9;No;1&amp;Q10;No;1&amp;Q11;No;1&amp;Q12;No;1&amp;Q13;No;1&amp;Q14;No;1&amp;Q15;No;1&amp;Q16;No;1&amp;Q17;No;1&amp;Q18;Yes;0.25&amp;Q19;Yes;0.25&amp;Q20;Yes;0.25&amp;Q21;Yes;0.25&amp;Q22;Yes;1&amp;Q23;No;1&amp;Q24;No;1&amp;Q25;No;1&amp;Q26;No;1&amp;Q27;Yes;1&amp;Q28;Yes;1&amp;Q29;Yes;1&amp;Q30;Yes;1&amp;Q31;Partially;1&amp;Q32;No;1&amp;Q33;No;1&amp;Q34;Yes;1&amp;Q35;No;1&amp;Q36;No;1&amp;Q37;No;1&amp;Q38;No;1&amp;Q39;No;1&amp;Q40;No;1&amp;Q41;Yes;1&amp;Q42;No;1&amp;Q43;No;1&amp;Q44;Yes;1&amp;Q45;No;1&amp;Q46;No;1</v>
+        <v>Q1;Yes;1&amp;Q2;Yes;1&amp;Q3;Yes;1&amp;Q4;Partially;1&amp;Q5;Yes;1&amp;Q6;No;1&amp;Q7;Yes;1&amp;Q8;Yes;1&amp;Q9;No;1&amp;Q10;No;1&amp;Q11;No;1&amp;Q12;No;1&amp;Q13;No;1&amp;Q14;No;1&amp;Q15;No;1&amp;Q16;No;1&amp;Q17;No;1&amp;Q18;Yes;0.25&amp;Q19;No;0.25&amp;Q20;No;0.25&amp;Q21;No;0.25&amp;Q22;No;1&amp;Q23;No;1&amp;Q24;No;1&amp;Q25;No;1&amp;Q26;No;1&amp;Q27;Yes;1&amp;Q28;Yes;1&amp;Q29;Yes;1&amp;Q30;Yes;1&amp;Q31;Partially;1&amp;Q32;No;1&amp;Q33;No;1&amp;Q34;Yes;1&amp;Q35;No;1&amp;Q36;No;1&amp;Q37;No;1&amp;Q38;No;1&amp;Q39;No;1&amp;Q40;No;1&amp;Q41;Yes;1&amp;Q42;No;1&amp;Q43;No;1&amp;Q44;Yes;1&amp;Q45;No;1&amp;Q46;No;1</v>
       </c>
       <c r="C10" s="19"/>
       <c r="D10" s="20"/>
@@ -1687,7 +1687,7 @@
         <v>47</v>
       </c>
       <c r="E33" s="26" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F33" s="26"/>
       <c r="G33" s="26"/>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="K33" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J33,E33,H33)</f>
-        <v>Q19;Yes;0.25</v>
+        <v>Q19;No;0.25</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1714,7 +1714,7 @@
         <v>48</v>
       </c>
       <c r="E34" s="29" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F34" s="29"/>
       <c r="G34" s="29"/>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="K34" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J34,E34,H34)</f>
-        <v>Q20;Yes;0.25</v>
+        <v>Q20;No;0.25</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1741,7 +1741,7 @@
         <v>49</v>
       </c>
       <c r="E35" s="26" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F35" s="26"/>
       <c r="G35" s="26"/>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="K35" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J35,E35,H35)</f>
-        <v>Q21;Yes;0.25</v>
+        <v>Q21;No;0.25</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1768,7 +1768,7 @@
         <v>50</v>
       </c>
       <c r="E36" s="29" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F36" s="29"/>
       <c r="G36" s="29"/>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="K36" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J36,E36,H36)</f>
-        <v>Q22;Yes;1</v>
+        <v>Q22;No;1</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>